<commit_message>
Rename tube laser series to TubeCut Double Chuck / TubeCut Triple Chuck branding
</commit_message>
<xml_diff>
--- a/documentation/datasheets/Wavlon_Tube_Laser_Model_Matrix.xlsx
+++ b/documentation/datasheets/Wavlon_Tube_Laser_Model_Matrix.xlsx
@@ -17,10 +17,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="173">
   <si>
-    <t>Wavlon Tube Laser Series — Model Lineup</t>
-  </si>
-  <si>
-    <t>Full line-up: WV-T2 (Double Chuck) &amp; WV-T3 (Triple Chuck Heavy Duty)</t>
+    <t>Wavlon TubeCut Series — Model Lineup</t>
+  </si>
+  <si>
+    <t>Full line-up: TubeCut Double Chuck &amp; TubeCut Triple Chuck (Heavy Duty)</t>
   </si>
   <si>
     <t>Model</t>
@@ -50,10 +50,10 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>WV-T2-120</t>
-  </si>
-  <si>
-    <t>WV-T2</t>
+    <t>TDC-120</t>
+  </si>
+  <si>
+    <t>TubeCut Double Chuck</t>
   </si>
   <si>
     <t>Entry</t>
@@ -71,7 +71,7 @@
     <t/>
   </si>
   <si>
-    <t>WV-T2-160</t>
+    <t>TDC-160</t>
   </si>
   <si>
     <t>160 mm</t>
@@ -83,7 +83,7 @@
     <t>Popular</t>
   </si>
   <si>
-    <t>WV-T2-240</t>
+    <t>TDC-240</t>
   </si>
   <si>
     <t>Intermediate</t>
@@ -95,7 +95,7 @@
     <t>4 / 6 / 8 kW</t>
   </si>
   <si>
-    <t>WV-T2-360</t>
+    <t>TDC-360</t>
   </si>
   <si>
     <t>360 mm</t>
@@ -104,10 +104,10 @@
     <t>6 / 8 / 12 kW</t>
   </si>
   <si>
-    <t>WV-T3-360</t>
-  </si>
-  <si>
-    <t>WV-T3</t>
+    <t>TTC-360</t>
+  </si>
+  <si>
+    <t>TubeCut Triple Chuck</t>
   </si>
   <si>
     <t>Heavy Duty</t>
@@ -116,7 +116,7 @@
     <t>12,000 mm</t>
   </si>
   <si>
-    <t>WV-T3-520</t>
+    <t>TTC-520</t>
   </si>
   <si>
     <t>520 mm</t>
@@ -125,7 +125,7 @@
     <t>12 / 16 / 20 kW</t>
   </si>
   <si>
-    <t>WV-T3-680</t>
+    <t>TTC-680</t>
   </si>
   <si>
     <t>Heavy Duty (Max)</t>
@@ -152,7 +152,7 @@
     <t>Parameter</t>
   </si>
   <si>
-    <t>WV-T3-680/570</t>
+    <t>TTC-680/570</t>
   </si>
   <si>
     <t>Max diameter — round</t>
@@ -323,7 +323,7 @@
     <t>Standard Componentry &amp; Brand Sourcing</t>
   </si>
   <si>
-    <t>Applies across the full WV-T2 / WV-T3 line-up unless a model-specific substitution is required.</t>
+    <t>Applies across the full TubeCut Double Chuck / TubeCut Triple Chuck line-up unless a model-specific substitution is required.</t>
   </si>
   <si>
     <t>Component</t>
@@ -437,13 +437,13 @@
     <t>Loading System</t>
   </si>
   <si>
-    <t>Semi-Auto (WV-T2) / Full-Auto Pneumatic Roller (WV-T3)</t>
+    <t>Semi-Auto (TubeCut Double Chuck) / Full-Auto Pneumatic Roller (TubeCut Triple Chuck)</t>
   </si>
   <si>
     <t>LD Laser Cross-Reference</t>
   </si>
   <si>
-    <t>Maps each Wavlon model to its closest LD Laser (LONGDIAO) catalog equivalent.</t>
+    <t>Maps each Wavlon TubeCut model to its closest LD Laser (LONGDIAO) catalog equivalent.</t>
   </si>
   <si>
     <t>Wavlon Model</t>
@@ -524,13 +524,13 @@
     <t>Power tier options are proposed groupings within LD's stated 1.5–12kW (T5) and 6–30kW (T8) ranges — confirm exact discrete wattages available from Raycus/MAX before publishing external pricing.</t>
   </si>
   <si>
-    <t>Acceleration figure for WV-T3 (≈1.0G) is an engineering estimate; LD's T8 catalog page did not show a numeric acceleration value at time of extraction.</t>
-  </si>
-  <si>
-    <t>Machine footprint and gross weight for all models except WV-T2-120 are scaled estimates from the single grounded reference datasheet (S5-6012-3000W) — confirm with engineering before quoting.</t>
-  </si>
-  <si>
-    <t>WV-T3-680/570 flagship diameter was specified directly by Wavlon management and does not exactly match a single LD T8 catalog code (closest are 12064 / 12083).</t>
+    <t>Acceleration figure for TubeCut Triple Chuck (≈1.0G) is an engineering estimate; LD's T8 catalog page did not show a numeric acceleration value at time of extraction.</t>
+  </si>
+  <si>
+    <t>Machine footprint and gross weight for all models except TDC-120 are scaled estimates from the single grounded reference datasheet (S5-6012-3000W) — confirm with engineering before quoting.</t>
+  </si>
+  <si>
+    <t>TTC-680/570 flagship diameter was specified directly by Wavlon management and does not exactly match a single LD T8 catalog code (closest are 12064 / 12083).</t>
   </si>
   <si>
     <t>This workbook is an internal sales-engineering / quoting reference. Website and CRM (Lovable) entries should be created from this once figures are confirmed.</t>
@@ -1015,7 +1015,7 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="5" max="6" width="13" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>

</xml_diff>